<commit_message>
Fresh gold-project PDFs on the Mac after the Windows sync
The gold film was built and exported through the synced core (0 unexpected
failures, verification passed). Screenplay, Sides, call sheet, Day Out of Days
and budget pages were drawn and checked by eye against the v5 standard and the
PDF design package v2; notes and pictures in
docs/release/evidence/mac/windows-sync-2026-10-27/pdf-check/.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/gold-project/outputs/reports/cast_scene.xlsx
+++ b/tests/gold-project/outputs/reports/cast_scene.xlsx
@@ -40,7 +40,7 @@
     <t>3, 4, 5, 6, 7, 8, 9, 10, 11, 12, 13, 14, 15, 16, 17, 18, 19, 20, 21, 23, 25, 26, 27, 28, 29, 30, 32, 34, 36, 39, 40, 41, 42, 43, 44, 45</t>
   </si>
   <si>
-    <t>Shoot Day 12 · Sat 23 Jan 2027; Shoot Day 3 · Wed 13 Jan 2027; Shoot Day 4 · Thu 14 Jan 2027; Shoot Day 7 · Mon 18 Jan 2027; Shoot Day 10 · Thu 21 Jan 2027; Shoot Day 5 · Fri 15 Jan 2027; Shoot Day 2 · Tue 12 Jan 2027; Shoot Day 6 · Sat 16 Jan 2027; Shoot Day 11 · Fri 22 Jan 2027; Shoot Day 8 · Tue 19 Jan 2027; Shoot Day 1 · Mon 11 Jan 2027; Shoot Day 9 · Wed 20 Jan 2027; Shoot Day 14 · Tue 26 Jan 2027</t>
+    <t>Shoot Day 1 · Mon 11 Jan 2027; Shoot Day 2 · Tue 12 Jan 2027; Shoot Day 3 · Wed 13 Jan 2027; Shoot Day 4 · Thu 14 Jan 2027; Shoot Day 5 · Fri 15 Jan 2027; Shoot Day 6 · Sat 16 Jan 2027; Shoot Day 7 · Mon 18 Jan 2027; Shoot Day 8 · Tue 19 Jan 2027; Shoot Day 9 · Wed 20 Jan 2027; Shoot Day 10 · Thu 21 Jan 2027; Shoot Day 11 · Fri 22 Jan 2027; Shoot Day 12 · Sat 23 Jan 2027; Shoot Day 14 · Tue 26 Jan 2027</t>
   </si>
   <si>
     <t>K. P. Gopinathan</t>
@@ -52,7 +52,7 @@
     <t>5, 6, 10, 15, 25, 26, 39, 40, 42, 45</t>
   </si>
   <si>
-    <t>Shoot Day 3 · Wed 13 Jan 2027; Shoot Day 4 · Thu 14 Jan 2027; Shoot Day 8 · Tue 19 Jan 2027; Shoot Day 12 · Sat 23 Jan 2027; Shoot Day 9 · Wed 20 Jan 2027; Shoot Day 14 · Tue 26 Jan 2027</t>
+    <t>Shoot Day 3 · Wed 13 Jan 2027; Shoot Day 4 · Thu 14 Jan 2027; Shoot Day 8 · Tue 19 Jan 2027; Shoot Day 9 · Wed 20 Jan 2027; Shoot Day 12 · Sat 23 Jan 2027; Shoot Day 14 · Tue 26 Jan 2027</t>
   </si>
   <si>
     <t>Sabitha Rasheed</t>
@@ -64,7 +64,7 @@
     <t>3, 6, 9, 13, 14, 16, 18, 20, 21, 23, 24, 34, 38, 40, 42, 43</t>
   </si>
   <si>
-    <t>Shoot Day 12 · Sat 23 Jan 2027; Shoot Day 4 · Thu 14 Jan 2027; Shoot Day 5 · Fri 15 Jan 2027; Shoot Day 6 · Sat 16 Jan 2027; Shoot Day 10 · Thu 21 Jan 2027; Shoot Day 7 · Mon 18 Jan 2027; Shoot Day 8 · Tue 19 Jan 2027; Shoot Day 9 · Wed 20 Jan 2027; Shoot Day 14 · Tue 26 Jan 2027</t>
+    <t>Shoot Day 4 · Thu 14 Jan 2027; Shoot Day 5 · Fri 15 Jan 2027; Shoot Day 6 · Sat 16 Jan 2027; Shoot Day 7 · Mon 18 Jan 2027; Shoot Day 8 · Tue 19 Jan 2027; Shoot Day 9 · Wed 20 Jan 2027; Shoot Day 10 · Thu 21 Jan 2027; Shoot Day 12 · Sat 23 Jan 2027; Shoot Day 14 · Tue 26 Jan 2027</t>
   </si>
   <si>
     <t>Not cast yet</t>
@@ -97,7 +97,7 @@
     <t>2, 17, 29, 30, 31, 32, 33, 38, 40</t>
   </si>
   <si>
-    <t>Shoot Day 2 · Tue 12 Jan 2027; Shoot Day 5 · Fri 15 Jan 2027; Shoot Day 1 · Mon 11 Jan 2027; Shoot Day 11 · Fri 22 Jan 2027; Shoot Day 9 · Wed 20 Jan 2027</t>
+    <t>Shoot Day 1 · Mon 11 Jan 2027; Shoot Day 2 · Tue 12 Jan 2027; Shoot Day 5 · Fri 15 Jan 2027; Shoot Day 9 · Wed 20 Jan 2027; Shoot Day 11 · Fri 22 Jan 2027</t>
   </si>
   <si>
     <t>Reshmi Pillai</t>
@@ -109,7 +109,7 @@
     <t>5, 19, 31, 32, 40, 42</t>
   </si>
   <si>
-    <t>Shoot Day 3 · Wed 13 Jan 2027; Shoot Day 11 · Fri 22 Jan 2027; Shoot Day 9 · Wed 20 Jan 2027; Shoot Day 14 · Tue 26 Jan 2027</t>
+    <t>Shoot Day 3 · Wed 13 Jan 2027; Shoot Day 9 · Wed 20 Jan 2027; Shoot Day 11 · Fri 22 Jan 2027; Shoot Day 14 · Tue 26 Jan 2027</t>
   </si>
   <si>
     <t>Divya Mathew</t>
@@ -121,7 +121,7 @@
     <t>1, 2, 4, 10, 16, 19, 33, 34, 35, 40, 41</t>
   </si>
   <si>
-    <t>Shoot Day 13 · Mon 25 Jan 2027; Shoot Day 2 · Tue 12 Jan 2027; Shoot Day 12 · Sat 23 Jan 2027; Shoot Day 4 · Thu 14 Jan 2027; Shoot Day 6 · Sat 16 Jan 2027; Shoot Day 11 · Fri 22 Jan 2027; Shoot Day 9 · Wed 20 Jan 2027; Shoot Day 3 · Wed 13 Jan 2027</t>
+    <t>Shoot Day 2 · Tue 12 Jan 2027; Shoot Day 3 · Wed 13 Jan 2027; Shoot Day 4 · Thu 14 Jan 2027; Shoot Day 6 · Sat 16 Jan 2027; Shoot Day 9 · Wed 20 Jan 2027; Shoot Day 11 · Fri 22 Jan 2027; Shoot Day 12 · Sat 23 Jan 2027; Shoot Day 13 · Mon 25 Jan 2027</t>
   </si>
   <si>
     <t>Gauri Krishna</t>
@@ -175,7 +175,7 @@
     <t>9, 11, 12, 13, 14, 16, 21, 23, 28, 29, 34, 38, 40, 41, 43</t>
   </si>
   <si>
-    <t>Shoot Day 5 · Fri 15 Jan 2027; Shoot Day 2 · Tue 12 Jan 2027; Shoot Day 3 · Wed 13 Jan 2027; Shoot Day 6 · Sat 16 Jan 2027; Shoot Day 7 · Mon 18 Jan 2027; Shoot Day 8 · Tue 19 Jan 2027; Shoot Day 1 · Mon 11 Jan 2027; Shoot Day 9 · Wed 20 Jan 2027; Shoot Day 14 · Tue 26 Jan 2027</t>
+    <t>Shoot Day 1 · Mon 11 Jan 2027; Shoot Day 2 · Tue 12 Jan 2027; Shoot Day 3 · Wed 13 Jan 2027; Shoot Day 5 · Fri 15 Jan 2027; Shoot Day 6 · Sat 16 Jan 2027; Shoot Day 7 · Mon 18 Jan 2027; Shoot Day 8 · Tue 19 Jan 2027; Shoot Day 9 · Wed 20 Jan 2027; Shoot Day 14 · Tue 26 Jan 2027</t>
   </si>
   <si>
     <t>Karan Shetty</t>
@@ -199,7 +199,7 @@
     <t>7, 8, 18, 23, 25, 26, 27, 28, 29, 30, 36, 37, 38, 40, 42</t>
   </si>
   <si>
-    <t>Shoot Day 7 · Mon 18 Jan 2027; Shoot Day 10 · Thu 21 Jan 2027; Shoot Day 8 · Tue 19 Jan 2027; Shoot Day 12 · Sat 23 Jan 2027; Shoot Day 1 · Mon 11 Jan 2027; Shoot Day 5 · Fri 15 Jan 2027; Shoot Day 9 · Wed 20 Jan 2027; Shoot Day 14 · Tue 26 Jan 2027</t>
+    <t>Shoot Day 1 · Mon 11 Jan 2027; Shoot Day 5 · Fri 15 Jan 2027; Shoot Day 7 · Mon 18 Jan 2027; Shoot Day 8 · Tue 19 Jan 2027; Shoot Day 9 · Wed 20 Jan 2027; Shoot Day 10 · Thu 21 Jan 2027; Shoot Day 12 · Sat 23 Jan 2027; Shoot Day 14 · Tue 26 Jan 2027</t>
   </si>
   <si>
     <t>Thampi Cherian</t>
@@ -211,7 +211,7 @@
     <t>1, 34, 35, 36, 40</t>
   </si>
   <si>
-    <t>Shoot Day 13 · Mon 25 Jan 2027; Shoot Day 6 · Sat 16 Jan 2027; Shoot Day 10 · Thu 21 Jan 2027; Shoot Day 9 · Wed 20 Jan 2027</t>
+    <t>Shoot Day 6 · Sat 16 Jan 2027; Shoot Day 9 · Wed 20 Jan 2027; Shoot Day 10 · Thu 21 Jan 2027; Shoot Day 13 · Mon 25 Jan 2027</t>
   </si>
   <si>
     <t>Ameya Suresh</t>
@@ -884,7 +884,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="200" verticalDpi="200"/>
   <headerFooter>
-    <oddFooter>&amp;CCreated with OpenFrame Studio</oddFooter>
+    <oddFooter>&amp;CCreated using OpenFrame</oddFooter>
   </headerFooter>
 </worksheet>
 </file>
</xml_diff>